<commit_message>
Se agrega el 12 de abril DG
</commit_message>
<xml_diff>
--- a/reporte/base_HE_20260422.xlsx
+++ b/reporte/base_HE_20260422.xlsx
@@ -530,10 +530,10 @@
     <t xml:space="preserve">SB, JLC</t>
   </si>
   <si>
-    <t xml:space="preserve">OT # 174472. Yantzaza,se ejecuta Plan de Maniobras en coordinación con Centro de Control.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['1', '2', '4', '5']</t>
+    <t xml:space="preserve">OT # 174472. En Yantzaza se realiza plan de maniobras en coordinación con Centro de Control, segun WR..1103028506. cierre de seccionadores tipo barra en estructura: 211933, para enmallar AP Yantzaza III con Paquisha En estructura: 255182 apertura de seccionadores tipo barra para separar AP Yantzaza III con Paquisha, or cubrir carga por trabajo en S/E Bomboiza Traslado desde Yantzaza hasta Muchime En Muchime en reguladores de voltaje en coordinación con Centro de Control, se posesiona en Manual y se coloca el TAP en Neutral a los Reguladores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['2', '4', '5']</t>
   </si>
   <si>
     <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-10 (021) SB.pdf</t>
@@ -584,105 +584,99 @@
     <t xml:space="preserve">['17', '18', '19']</t>
   </si>
   <si>
-    <t xml:space="preserve">OT # 174867. Los Encuentros, se coordinan maniobras con Centro de Control</t>
+    <t xml:space="preserve">OT # 174867. Chimbutza, maniobras en coordinación con CC; Fall del AP Los Encuentros, se encuentra un deslizamiento de tierra de gran magnitud, Est 289767 colapsada. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">['2']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-16 (021) SB.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 174940. Loja – Yantzaza, sector Chimbutza se colabora con trabajos de aplomada de estructura y normalizar tipología del AP Los Encuentros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['8', '9', '10']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-17 (021) SB.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AA, AO, JLC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 174948. Chimbutza. aplomado de estructura 262666, cambio de 2 penos pin, enderezada de cruzatas, regulado de los tensores; maniobras en coordinación con CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['6', '8']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-17 (022) AA.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 175032. El Recreo, cambio de breaker de caja moldeada en mal estado Med # 290277. Guayabal, Est 35094, se rehabilita transformador 14001; Causa: líneas arrancadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REDES:60, ACOMETIDAS:20, MEDIDORES:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-18 (021) SB.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 175032.  La Libertad, acometida arrancada de Med # 124603; Causa: crecida de rio. Pita Alto, Med # 241722, acometida arrancada por vegetación, se repara. Barrio Central, Est 268537 se rehabilita trafo # 16229 de 50 KVA; Causa: RBV arrancada (1/0 ACSR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REDES:50, ACOMETIDAS:25, MEDIDORES:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3, 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 175048. Yantzaza,  Est 27383 impactada sobre vehículo liviano, por emergencia el cliente realiza el cambio de estructura de manera particular, se colabora en arreglo de medidores. Montalvo, Est 223650, se retira vegetación y cambi fusible de 0,7A-SR del Trafo # 22068.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['3', '5', '6', '7']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-19 (021) SB.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 175048. Ungumiatza, Est 29607 quebrada por caída de árbol seco en sus base (25 mts altura), se programa cambio. La Florida, arreglo de conexiones en Med # 18-252259.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REDES:70, MEDIDORES:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['10', '11', '13', '14', '15']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB, AO, GT, JLC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 175082. Ungumiatza, Izaje de estructura de 11R para restituir estructura en mal estado, empalme montado y regulado de LMV, se energiza y retorna a Yantzaza.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['7', '10']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-20 (021) SB.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT # 173844. Se Coordina trabajos con jefe inmediato y centro de control, se realiza maniobras de mallado interno del Reconectador Las Peñas con Nueva Tarqui y Neutralizada de Reguladores Gualaquiza.</t>
   </si>
   <si>
     <t xml:space="preserve">['1']</t>
   </si>
   <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-16 (021) SB.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 174867. Chimbutza, maniobras en coordinación con CC; Fall del AP Los Encuentros, se encuentra un deslizamiento de tierra de gran magnitud, Est 289767 colapsada. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">['2']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 174940. Loja – Yantzaza, sector Chimbutza se colabora con trabajos de aplomada de estructura y normalizar tipología del AP Los Encuentros.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['8', '9', '10']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-17 (021) SB.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AA, AO, JLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 174948. Chimbutza. aplomado de estructura 262666, cambio de 2 penos pin, enderezada de cruzatas, regulado de los tensores; maniobras en coordinación con CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['6', '8']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-17 (022) AA.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 175032. El Recreo, cambio de breaker de caja moldeada en mal estado Med # 290277. Guayabal, Est 35094, se rehabilita transformador 14001; Causa: líneas arrancadas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REDES:60, ACOMETIDAS:20, MEDIDORES:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1, 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-18 (021) SB.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 175032.  La Libertad, acometida arrancada de Med # 124603; Causa: crecida de rio. Pita Alto, Med # 241722, acometida arrancada por vegetación, se repara. Barrio Central, Est 268537 se rehabilita trafo # 16229 de 50 KVA; Causa: RBV arrancada (1/0 ACSR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REDES:50, ACOMETIDAS:25, MEDIDORES:25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3, 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 175048. Yantzaza,  Est 27383 impactada sobre vehículo liviano, por emergencia el cliente realiza el cambio de estructura de manera particular, se colabora en arreglo de medidores. Montalvo, Est 223650, se retira vegetación y cambi fusible de 0,7A-SR del Trafo # 22068.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['3', '5', '6', '7']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-19 (021) SB.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 175048. Ungumiatza, Est 29607 quebrada por caída de árbol seco en sus base (25 mts altura), se programa cambio. La Florida, arreglo de conexiones en Med # 18-252259.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REDES:70, MEDIDORES:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['10', '11', '13', '14', '15']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SB, AO, GT, JLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 175082. Ungumiatza, Izaje de estructura de 11R para restituir estructura en mal estado, empalme montado y regulado de LMV, se energiza y retorna a Yantzaza.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['7', '10']</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT [04] Cuadrilla Yantzaza 2026-04-20 (021) SB.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT # 173844. Se Coordina trabajos con jefe inmediato y centro de control, se realiza maniobras de mallado interno del Reconectador Las Peñas con Nueva Tarqui y Neutralizada de Reguladores Gualaquiza.</t>
-  </si>
-  <si>
     <t xml:space="preserve">OT [05] Energizados Yantzaza 2026-04-01 (027) LA.pdf</t>
   </si>
   <si>
@@ -770,6 +764,15 @@
     <t xml:space="preserve">OT [06] Cuadrilla Paquisha 2026-04-11 (036) DG.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">OT # 174581. San Luis, Est 270680 , se rehabilita transformador 24432; Causa: Sobrecarga. Zumbi, Med # 18-215893, se encuentra puentes y conector en malas condiciones, se corrige en cable preensamblado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">['1', '2', '3', '4', '5']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT [06] Cuadrilla Paquisha 2026-04-12 (036) DG.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">JA, DG, MS,  JJ</t>
   </si>
   <si>
@@ -1188,9 +1191,6 @@
   </si>
   <si>
     <t xml:space="preserve">OT # 174080. DIA FESTIVO “Viernes Santo” Naichap, Est 037299, revision y restitucion medidor 194238 por 18-258039 borneras quemadas. Aguacate, Est 127921, revision y restitucion medidor 194324 por 18-258040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">['1', '2', '3', '4', '5']</t>
   </si>
   <si>
     <t xml:space="preserve">OT [24] Agencia Gualaquiza 2026-04-03 (061) CB.pdf</t>
@@ -3060,7 +3060,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
         <v>49</v>
       </c>
@@ -3569,14 +3569,14 @@
         <v>46122</v>
       </c>
       <c r="E27" s="29" t="n">
-        <v>0.270833333333333</v>
+        <v>0.28125</v>
       </c>
       <c r="F27" s="29" t="n">
         <v>0.333333333333333</v>
       </c>
       <c r="G27" s="21" t="n">
         <f aca="false">F27-E27</f>
-        <v>0.0625</v>
+        <v>0.0520833333333333</v>
       </c>
       <c r="H27" s="32" t="s">
         <v>168</v>
@@ -3591,7 +3591,7 @@
         <v>169</v>
       </c>
       <c r="L27" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M27" s="31" t="s">
         <v>170</v>
@@ -3839,14 +3839,14 @@
         <v>46128</v>
       </c>
       <c r="E33" s="29" t="n">
-        <v>0.231944444444445</v>
+        <v>0.25</v>
       </c>
       <c r="F33" s="29" t="n">
-        <v>0.249305555555556</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G33" s="21" t="n">
         <f aca="false">F33-E33</f>
-        <v>0.0173611111111111</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="H33" s="32" t="s">
         <v>186</v>
@@ -3867,7 +3867,7 @@
         <v>188</v>
       </c>
       <c r="N33" s="31" t="s">
-        <v>189</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3875,23 +3875,23 @@
         <v>54</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>130</v>
+        <v>83</v>
       </c>
       <c r="D34" s="28" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="E34" s="29" t="n">
-        <v>0.25</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F34" s="29" t="n">
-        <v>0.333333333333333</v>
+        <v>0.8125</v>
       </c>
       <c r="G34" s="21" t="n">
         <f aca="false">F34-E34</f>
-        <v>0.0833333333333333</v>
+        <v>0.104166666666667</v>
       </c>
       <c r="H34" s="32" t="s">
         <v>190</v>
@@ -3900,16 +3900,16 @@
         <v>79</v>
       </c>
       <c r="J34" s="31" t="n">
-        <v>174867</v>
+        <v>174940</v>
       </c>
       <c r="K34" s="31" t="s">
         <v>191</v>
       </c>
       <c r="L34" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M34" s="31" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="N34" s="31" t="s">
         <v>82</v>
@@ -3920,7 +3920,7 @@
         <v>54</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C35" s="27" t="s">
         <v>83</v>
@@ -3939,22 +3939,22 @@
         <v>0.104166666666667</v>
       </c>
       <c r="H35" s="32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I35" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J35" s="31" t="n">
-        <v>174940</v>
+        <v>174948</v>
       </c>
       <c r="K35" s="31" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L35" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M35" s="31" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="N35" s="31" t="s">
         <v>82</v>
@@ -3965,19 +3965,19 @@
         <v>54</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>196</v>
+        <v>167</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="D36" s="28" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="E36" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="F36" s="29" t="n">
-        <v>0.8125</v>
+        <v>0.541666666666667</v>
       </c>
       <c r="G36" s="21" t="n">
         <f aca="false">F36-E36</f>
@@ -3987,22 +3987,22 @@
         <v>197</v>
       </c>
       <c r="I36" s="31" t="s">
-        <v>79</v>
+        <v>198</v>
       </c>
       <c r="J36" s="31" t="n">
-        <v>174948</v>
+        <v>175032</v>
       </c>
       <c r="K36" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L36" s="31" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="M36" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="N36" s="31" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4019,32 +4019,32 @@
         <v>46130</v>
       </c>
       <c r="E37" s="29" t="n">
-        <v>0.4375</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="F37" s="29" t="n">
-        <v>0.541666666666667</v>
+        <v>0.847222222222222</v>
       </c>
       <c r="G37" s="21" t="n">
         <f aca="false">F37-E37</f>
-        <v>0.104166666666667</v>
+        <v>0.263888888888889</v>
       </c>
       <c r="H37" s="30" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I37" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J37" s="31" t="n">
         <v>175032</v>
       </c>
       <c r="K37" s="31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L37" s="31" t="n">
         <v>10</v>
       </c>
       <c r="M37" s="31" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="N37" s="31" t="s">
         <v>95</v>
@@ -4058,38 +4058,38 @@
         <v>167</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D38" s="28" t="n">
-        <v>46130</v>
+        <v>46131</v>
       </c>
       <c r="E38" s="29" t="n">
-        <v>0.583333333333333</v>
+        <v>0.28125</v>
       </c>
       <c r="F38" s="29" t="n">
-        <v>0.847222222222222</v>
+        <v>0.548611111111111</v>
       </c>
       <c r="G38" s="21" t="n">
         <f aca="false">F38-E38</f>
-        <v>0.263888888888889</v>
+        <v>0.267361111111111</v>
       </c>
       <c r="H38" s="30" t="s">
         <v>204</v>
       </c>
       <c r="I38" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="J38" s="31" t="n">
+        <v>175048</v>
+      </c>
+      <c r="K38" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="J38" s="31" t="n">
-        <v>175032</v>
-      </c>
-      <c r="K38" s="31" t="s">
+      <c r="L38" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="M38" s="31" t="s">
         <v>206</v>
-      </c>
-      <c r="L38" s="31" t="n">
-        <v>10</v>
-      </c>
-      <c r="M38" s="31" t="s">
-        <v>203</v>
       </c>
       <c r="N38" s="31" t="s">
         <v>95</v>
@@ -4109,32 +4109,32 @@
         <v>46131</v>
       </c>
       <c r="E39" s="29" t="n">
-        <v>0.28125</v>
+        <v>0.696527777777778</v>
       </c>
       <c r="F39" s="29" t="n">
-        <v>0.548611111111111</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="G39" s="21" t="n">
         <f aca="false">F39-E39</f>
-        <v>0.267361111111111</v>
+        <v>0.0951388888888889</v>
       </c>
       <c r="H39" s="30" t="s">
         <v>207</v>
       </c>
       <c r="I39" s="31" t="s">
-        <v>79</v>
+        <v>208</v>
       </c>
       <c r="J39" s="31" t="n">
         <v>175048</v>
       </c>
       <c r="K39" s="31" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L39" s="31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M39" s="31" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="N39" s="31" t="s">
         <v>95</v>
@@ -4145,86 +4145,86 @@
         <v>54</v>
       </c>
       <c r="B40" s="26" t="s">
-        <v>167</v>
+        <v>210</v>
       </c>
       <c r="C40" s="27" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="D40" s="28" t="n">
-        <v>46131</v>
+        <v>46132</v>
       </c>
       <c r="E40" s="29" t="n">
-        <v>0.696527777777778</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F40" s="29" t="n">
-        <v>0.791666666666667</v>
+        <v>0.784722222222222</v>
       </c>
       <c r="G40" s="21" t="n">
         <f aca="false">F40-E40</f>
-        <v>0.0951388888888889</v>
+        <v>0.0763888888888889</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="I40" s="31" t="s">
-        <v>211</v>
+        <v>79</v>
       </c>
       <c r="J40" s="31" t="n">
-        <v>175048</v>
+        <v>175082</v>
       </c>
       <c r="K40" s="31" t="s">
         <v>212</v>
       </c>
       <c r="L40" s="31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M40" s="31" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="N40" s="31" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>118</v>
+        <v>77</v>
       </c>
       <c r="D41" s="28" t="n">
-        <v>46132</v>
+        <v>46113</v>
       </c>
       <c r="E41" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.270833333333333</v>
       </c>
       <c r="F41" s="29" t="n">
-        <v>0.784722222222222</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G41" s="21" t="n">
         <f aca="false">F41-E41</f>
-        <v>0.0763888888888889</v>
+        <v>0.0625</v>
       </c>
       <c r="H41" s="30" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="I41" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J41" s="31" t="n">
-        <v>175082</v>
+        <v>173844</v>
       </c>
       <c r="K41" s="31" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="L41" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M41" s="31" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N41" s="31" t="s">
         <v>82</v>
@@ -4235,7 +4235,7 @@
         <v>55</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C42" s="27" t="s">
         <v>77</v>
@@ -4244,10 +4244,10 @@
         <v>46113</v>
       </c>
       <c r="E42" s="29" t="n">
-        <v>0.270833333333333</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F42" s="29" t="n">
-        <v>0.333333333333333</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="G42" s="21" t="n">
         <f aca="false">F42-E42</f>
@@ -4263,30 +4263,30 @@
         <v>173844</v>
       </c>
       <c r="K42" s="31" t="s">
-        <v>187</v>
+        <v>219</v>
       </c>
       <c r="L42" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M42" s="31" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="N42" s="31" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="28.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="26" t="s">
         <v>55</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="D43" s="28" t="n">
-        <v>46113</v>
+        <v>46118</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0.708333333333333</v>
@@ -4305,16 +4305,16 @@
         <v>79</v>
       </c>
       <c r="J43" s="31" t="n">
-        <v>173844</v>
+        <v>174118</v>
       </c>
       <c r="K43" s="31" t="s">
         <v>221</v>
       </c>
       <c r="L43" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M43" s="31" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="N43" s="31" t="s">
         <v>82</v>
@@ -4325,38 +4325,38 @@
         <v>55</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>118</v>
+        <v>77</v>
       </c>
       <c r="D44" s="28" t="n">
-        <v>46118</v>
+        <v>46127</v>
       </c>
       <c r="E44" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.28125</v>
       </c>
       <c r="F44" s="29" t="n">
-        <v>0.770833333333333</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G44" s="21" t="n">
         <f aca="false">F44-E44</f>
-        <v>0.0625</v>
+        <v>0.0520833333333333</v>
       </c>
       <c r="H44" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I44" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J44" s="31" t="n">
-        <v>174118</v>
+        <v>174761</v>
       </c>
       <c r="K44" s="31" t="s">
-        <v>223</v>
+        <v>151</v>
       </c>
       <c r="L44" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M44" s="31" t="s">
         <v>224</v>
@@ -4370,7 +4370,7 @@
         <v>55</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C45" s="27" t="s">
         <v>77</v>
@@ -4379,14 +4379,14 @@
         <v>46127</v>
       </c>
       <c r="E45" s="29" t="n">
-        <v>0.28125</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F45" s="29" t="n">
-        <v>0.333333333333333</v>
+        <v>0.8125</v>
       </c>
       <c r="G45" s="21" t="n">
         <f aca="false">F45-E45</f>
-        <v>0.0520833333333333</v>
+        <v>0.104166666666667</v>
       </c>
       <c r="H45" s="32" t="s">
         <v>225</v>
@@ -4398,58 +4398,58 @@
         <v>174761</v>
       </c>
       <c r="K45" s="31" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="L45" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M45" s="31" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="N45" s="31" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="26" t="s">
         <v>55</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="D46" s="28" t="n">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="E46" s="29" t="n">
         <v>0.708333333333333</v>
       </c>
       <c r="F46" s="29" t="n">
-        <v>0.8125</v>
+        <v>0.75</v>
       </c>
       <c r="G46" s="21" t="n">
         <f aca="false">F46-E46</f>
-        <v>0.104166666666667</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="H46" s="32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I46" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J46" s="31" t="n">
-        <v>174761</v>
+        <v>175038</v>
       </c>
       <c r="K46" s="31" t="s">
-        <v>194</v>
+        <v>227</v>
       </c>
       <c r="L46" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M46" s="31" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N46" s="31" t="s">
         <v>82</v>
@@ -4457,47 +4457,47 @@
     </row>
     <row r="47" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="26" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>118</v>
+        <v>9</v>
       </c>
       <c r="D47" s="28" t="n">
-        <v>46132</v>
+        <v>46116</v>
       </c>
       <c r="E47" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.431944444444445</v>
       </c>
       <c r="F47" s="29" t="n">
-        <v>0.75</v>
+        <v>0.475694444444444</v>
       </c>
       <c r="G47" s="21" t="n">
         <f aca="false">F47-E47</f>
-        <v>0.0416666666666667</v>
+        <v>0.04375</v>
       </c>
       <c r="H47" s="32" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I47" s="31" t="s">
-        <v>79</v>
+        <v>173</v>
       </c>
       <c r="J47" s="31" t="n">
-        <v>175038</v>
+        <v>174048</v>
       </c>
       <c r="K47" s="31" t="s">
-        <v>229</v>
+        <v>93</v>
       </c>
       <c r="L47" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M47" s="31" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="N47" s="31" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4505,23 +4505,23 @@
         <v>57</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D48" s="28" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="E48" s="29" t="n">
-        <v>0.431944444444445</v>
+        <v>0.638194444444444</v>
       </c>
       <c r="F48" s="29" t="n">
-        <v>0.475694444444444</v>
+        <v>0.688194444444444</v>
       </c>
       <c r="G48" s="21" t="n">
         <f aca="false">F48-E48</f>
-        <v>0.04375</v>
+        <v>0.05</v>
       </c>
       <c r="H48" s="32" t="s">
         <v>232</v>
@@ -4530,10 +4530,10 @@
         <v>173</v>
       </c>
       <c r="J48" s="31" t="n">
-        <v>174048</v>
+        <v>174127</v>
       </c>
       <c r="K48" s="31" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="L48" s="31" t="n">
         <v>3</v>
@@ -4550,44 +4550,44 @@
         <v>57</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C49" s="27" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
       <c r="D49" s="28" t="n">
-        <v>46117</v>
+        <v>46121</v>
       </c>
       <c r="E49" s="29" t="n">
-        <v>0.638194444444444</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F49" s="29" t="n">
-        <v>0.688194444444444</v>
+        <v>0.8125</v>
       </c>
       <c r="G49" s="21" t="n">
         <f aca="false">F49-E49</f>
-        <v>0.05</v>
+        <v>0.104166666666667</v>
       </c>
       <c r="H49" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I49" s="31" t="s">
-        <v>173</v>
+        <v>79</v>
       </c>
       <c r="J49" s="31" t="n">
-        <v>174127</v>
+        <v>174423</v>
       </c>
       <c r="K49" s="31" t="s">
-        <v>148</v>
+        <v>236</v>
       </c>
       <c r="L49" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M49" s="31" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="N49" s="31" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4595,38 +4595,38 @@
         <v>57</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>130</v>
+        <v>83</v>
       </c>
       <c r="D50" s="28" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="E50" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.25</v>
       </c>
       <c r="F50" s="29" t="n">
-        <v>0.8125</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G50" s="21" t="n">
         <f aca="false">F50-E50</f>
-        <v>0.104166666666667</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="H50" s="31" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I50" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J50" s="31" t="n">
-        <v>174423</v>
+        <v>174471</v>
       </c>
       <c r="K50" s="31" t="s">
-        <v>238</v>
+        <v>93</v>
       </c>
       <c r="L50" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M50" s="31" t="s">
         <v>239</v>
@@ -4640,7 +4640,7 @@
         <v>57</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C51" s="27" t="s">
         <v>83</v>
@@ -4649,32 +4649,32 @@
         <v>46122</v>
       </c>
       <c r="E51" s="29" t="n">
-        <v>0.25</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="F51" s="29" t="n">
-        <v>0.333333333333333</v>
+        <v>0.75</v>
       </c>
       <c r="G51" s="21" t="n">
         <f aca="false">F51-E51</f>
-        <v>0.0833333333333333</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="H51" s="31" t="s">
         <v>240</v>
       </c>
       <c r="I51" s="31" t="s">
-        <v>79</v>
+        <v>173</v>
       </c>
       <c r="J51" s="31" t="n">
         <v>174471</v>
       </c>
       <c r="K51" s="31" t="s">
-        <v>93</v>
+        <v>241</v>
       </c>
       <c r="L51" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M51" s="31" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="N51" s="31" t="s">
         <v>82</v>
@@ -4685,44 +4685,44 @@
         <v>57</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="D52" s="28" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="E52" s="29" t="n">
-        <v>0.708333333333333</v>
+        <v>0.55625</v>
       </c>
       <c r="F52" s="29" t="n">
-        <v>0.75</v>
+        <v>0.709722222222222</v>
       </c>
       <c r="G52" s="21" t="n">
         <f aca="false">F52-E52</f>
-        <v>0.0416666666666667</v>
+        <v>0.153472222222222</v>
       </c>
       <c r="H52" s="31" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I52" s="31" t="s">
-        <v>173</v>
+        <v>79</v>
       </c>
       <c r="J52" s="31" t="n">
-        <v>174471</v>
+        <v>174548</v>
       </c>
       <c r="K52" s="31" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L52" s="31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M52" s="31" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="N52" s="31" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4730,41 +4730,41 @@
         <v>57</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D53" s="28" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="E53" s="29" t="n">
-        <v>0.55625</v>
+        <v>0.586111111111111</v>
       </c>
       <c r="F53" s="29" t="n">
-        <v>0.709722222222222</v>
+        <v>0.682638888888889</v>
       </c>
       <c r="G53" s="21" t="n">
         <f aca="false">F53-E53</f>
-        <v>0.153472222222222</v>
+        <v>0.0965277777777778</v>
       </c>
       <c r="H53" s="31" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I53" s="31" t="s">
         <v>79</v>
       </c>
       <c r="J53" s="31" t="n">
-        <v>174548</v>
+        <v>174581</v>
       </c>
       <c r="K53" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L53" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M53" s="31" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="N53" s="31" t="s">
         <v>95</v>
@@ -4775,7 +4775,7 @@
         <v>57</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C54" s="27" t="s">
         <v>77</v>
@@ -4794,7 +4794,7 @@
         <v>0.0416666666666667</v>
       </c>
       <c r="H54" s="31" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I54" s="31" t="s">
         <v>79</v>
@@ -4809,7 +4809,7 @@
         <v>2</v>
       </c>
       <c r="M54" s="31" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="N54" s="31" t="s">
         <v>82</v>
@@ -4820,7 +4820,7 @@
         <v>57</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C55" s="27" t="s">
         <v>77</v>
@@ -4839,7 +4839,7 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="H55" s="31" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I55" s="31" t="s">
         <v>79</v>
@@ -4848,13 +4848,13 @@
         <v>174770</v>
       </c>
       <c r="K55" s="31" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L55" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M55" s="31" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="N55" s="31" t="s">
         <v>82</v>
@@ -4865,7 +4865,7 @@
         <v>57</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C56" s="27" t="s">
         <v>9</v>
@@ -4884,7 +4884,7 @@
         <v>0.157638888888889</v>
       </c>
       <c r="H56" s="31" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I56" s="31" t="s">
         <v>79</v>
@@ -4893,13 +4893,13 @@
         <v>174999</v>
       </c>
       <c r="K56" s="31" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L56" s="31" t="n">
         <v>6</v>
       </c>
       <c r="M56" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N56" s="31" t="s">
         <v>95</v>
@@ -4910,7 +4910,7 @@
         <v>57</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C57" s="27" t="s">
         <v>11</v>
@@ -4929,7 +4929,7 @@
         <v>0.0444444444444444</v>
       </c>
       <c r="H57" s="31" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I57" s="31" t="s">
         <v>79</v>
@@ -4944,7 +4944,7 @@
         <v>3</v>
       </c>
       <c r="M57" s="31" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="N57" s="31" t="s">
         <v>95</v>
@@ -4955,7 +4955,7 @@
         <v>58</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C58" s="27" t="s">
         <v>130</v>
@@ -4974,7 +4974,7 @@
         <v>0.0625</v>
       </c>
       <c r="H58" s="31" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="I58" s="31" t="s">
         <v>79</v>
@@ -4983,13 +4983,13 @@
         <v>174393</v>
       </c>
       <c r="K58" s="31" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L58" s="31" t="n">
         <v>1</v>
       </c>
       <c r="M58" s="31" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="N58" s="31" t="s">
         <v>82</v>
@@ -5000,7 +5000,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C59" s="27" t="s">
         <v>130</v>
@@ -5019,7 +5019,7 @@
         <v>0.0458333333333333</v>
       </c>
       <c r="H59" s="31" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I59" s="31" t="s">
         <v>79</v>
@@ -5028,13 +5028,13 @@
         <v>174393</v>
       </c>
       <c r="K59" s="31" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L59" s="31" t="n">
         <v>1</v>
       </c>
       <c r="M59" s="31" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="N59" s="31" t="s">
         <v>82</v>
@@ -5045,7 +5045,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C60" s="27" t="s">
         <v>83</v>
@@ -5064,7 +5064,7 @@
         <v>0.0486111111111111</v>
       </c>
       <c r="H60" s="31" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I60" s="31" t="s">
         <v>79</v>
@@ -5073,13 +5073,13 @@
         <v>174473</v>
       </c>
       <c r="K60" s="31" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L60" s="31" t="n">
         <v>1</v>
       </c>
       <c r="M60" s="31" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N60" s="31" t="s">
         <v>82</v>
@@ -5090,7 +5090,7 @@
         <v>58</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C61" s="27" t="s">
         <v>83</v>
@@ -5109,7 +5109,7 @@
         <v>0.164583333333333</v>
       </c>
       <c r="H61" s="31" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I61" s="31" t="s">
         <v>79</v>
@@ -5124,7 +5124,7 @@
         <v>2</v>
       </c>
       <c r="M61" s="31" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="N61" s="31" t="s">
         <v>82</v>
@@ -5135,7 +5135,7 @@
         <v>58</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C62" s="27" t="s">
         <v>77</v>
@@ -5154,7 +5154,7 @@
         <v>0.0402777777777778</v>
       </c>
       <c r="H62" s="31" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I62" s="31" t="s">
         <v>79</v>
@@ -5169,7 +5169,7 @@
         <v>3</v>
       </c>
       <c r="M62" s="31" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N62" s="31" t="s">
         <v>82</v>
@@ -5180,7 +5180,7 @@
         <v>58</v>
       </c>
       <c r="B63" s="26" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C63" s="27" t="s">
         <v>77</v>
@@ -5199,7 +5199,7 @@
         <v>0.09375</v>
       </c>
       <c r="H63" s="31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I63" s="31" t="s">
         <v>89</v>
@@ -5214,7 +5214,7 @@
         <v>2</v>
       </c>
       <c r="M63" s="31" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N63" s="31" t="s">
         <v>82</v>
@@ -5225,7 +5225,7 @@
         <v>58</v>
       </c>
       <c r="B64" s="26" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C64" s="27" t="s">
         <v>11</v>
@@ -5244,22 +5244,22 @@
         <v>0.161111111111111</v>
       </c>
       <c r="H64" s="31" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I64" s="31" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J64" s="31" t="n">
         <v>175050</v>
       </c>
       <c r="K64" s="31" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="L64" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M64" s="31" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="N64" s="31" t="s">
         <v>95</v>
@@ -5270,7 +5270,7 @@
         <v>59</v>
       </c>
       <c r="B65" s="26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C65" s="27" t="s">
         <v>77</v>
@@ -5289,7 +5289,7 @@
         <v>0.0465277777777778</v>
       </c>
       <c r="H65" s="31" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="I65" s="31" t="s">
         <v>79</v>
@@ -5298,13 +5298,13 @@
         <v>173908</v>
       </c>
       <c r="K65" s="31" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="L65" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M65" s="31" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="N65" s="31" t="s">
         <v>82</v>
@@ -5315,7 +5315,7 @@
         <v>59</v>
       </c>
       <c r="B66" s="26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C66" s="27" t="s">
         <v>130</v>
@@ -5334,7 +5334,7 @@
         <v>0.0201388888888889</v>
       </c>
       <c r="H66" s="31" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I66" s="31" t="s">
         <v>79</v>
@@ -5343,13 +5343,13 @@
         <v>173951</v>
       </c>
       <c r="K66" s="31" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L66" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M66" s="31" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N66" s="31" t="s">
         <v>82</v>
@@ -5360,7 +5360,7 @@
         <v>59</v>
       </c>
       <c r="B67" s="26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C67" s="27" t="s">
         <v>83</v>
@@ -5379,7 +5379,7 @@
         <v>0.0319444444444444</v>
       </c>
       <c r="H67" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I67" s="31" t="s">
         <v>79</v>
@@ -5394,7 +5394,7 @@
         <v>3</v>
       </c>
       <c r="M67" s="31" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N67" s="31" t="s">
         <v>87</v>
@@ -5405,7 +5405,7 @@
         <v>59</v>
       </c>
       <c r="B68" s="26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C68" s="27" t="s">
         <v>11</v>
@@ -5424,7 +5424,7 @@
         <v>0.191666666666667</v>
       </c>
       <c r="H68" s="32" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I68" s="31" t="s">
         <v>79</v>
@@ -5433,13 +5433,13 @@
         <v>174070</v>
       </c>
       <c r="K68" s="31" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L68" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M68" s="31" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="N68" s="31" t="s">
         <v>95</v>
@@ -5450,7 +5450,7 @@
         <v>59</v>
       </c>
       <c r="B69" s="26" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C69" s="27" t="s">
         <v>9</v>
@@ -5469,22 +5469,22 @@
         <v>0.199305555555556</v>
       </c>
       <c r="H69" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I69" s="31" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J69" s="31" t="n">
         <v>174595</v>
       </c>
       <c r="K69" s="31" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L69" s="31" t="n">
         <v>9</v>
       </c>
       <c r="M69" s="31" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="N69" s="31" t="s">
         <v>95</v>
@@ -5495,7 +5495,7 @@
         <v>59</v>
       </c>
       <c r="B70" s="26" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C70" s="27" t="s">
         <v>11</v>
@@ -5514,7 +5514,7 @@
         <v>0.204861111111111</v>
       </c>
       <c r="H70" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I70" s="31" t="s">
         <v>79</v>
@@ -5523,13 +5523,13 @@
         <v>174643</v>
       </c>
       <c r="K70" s="31" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L70" s="31" t="n">
         <v>9</v>
       </c>
       <c r="M70" s="31" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="N70" s="31" t="s">
         <v>95</v>
@@ -5540,7 +5540,7 @@
         <v>59</v>
       </c>
       <c r="B71" s="26" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C71" s="27" t="s">
         <v>118</v>
@@ -5559,7 +5559,7 @@
         <v>0.0923611111111111</v>
       </c>
       <c r="H71" s="30" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I71" s="31" t="s">
         <v>79</v>
@@ -5574,7 +5574,7 @@
         <v>3</v>
       </c>
       <c r="M71" s="31" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N71" s="31" t="s">
         <v>82</v>
@@ -5585,7 +5585,7 @@
         <v>59</v>
       </c>
       <c r="B72" s="26" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C72" s="27" t="s">
         <v>9</v>
@@ -5604,7 +5604,7 @@
         <v>0.171527777777778</v>
       </c>
       <c r="H72" s="32" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I72" s="31" t="s">
         <v>79</v>
@@ -5613,13 +5613,13 @@
         <v>175002</v>
       </c>
       <c r="K72" s="31" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L72" s="31" t="n">
         <v>8</v>
       </c>
       <c r="M72" s="31" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="N72" s="31" t="s">
         <v>95</v>
@@ -5630,7 +5630,7 @@
         <v>59</v>
       </c>
       <c r="B73" s="26" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C73" s="27" t="s">
         <v>11</v>
@@ -5649,7 +5649,7 @@
         <v>0.122222222222222</v>
       </c>
       <c r="H73" s="31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="I73" s="31" t="s">
         <v>79</v>
@@ -5658,13 +5658,13 @@
         <v>175025</v>
       </c>
       <c r="K73" s="31" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L73" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M73" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="N73" s="31" t="s">
         <v>95</v>
@@ -5675,7 +5675,7 @@
         <v>61</v>
       </c>
       <c r="B74" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C74" s="27" t="s">
         <v>118</v>
@@ -5694,7 +5694,7 @@
         <v>0.0868055555555556</v>
       </c>
       <c r="H74" s="32" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I74" s="31" t="s">
         <v>89</v>
@@ -5709,7 +5709,7 @@
         <v>3</v>
       </c>
       <c r="M74" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="N74" s="31" t="s">
         <v>82</v>
@@ -5720,7 +5720,7 @@
         <v>61</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C75" s="27" t="s">
         <v>113</v>
@@ -5739,7 +5739,7 @@
         <v>0.0972222222222222</v>
       </c>
       <c r="H75" s="32" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="I75" s="31" t="s">
         <v>79</v>
@@ -5754,7 +5754,7 @@
         <v>3</v>
       </c>
       <c r="M75" s="31" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="N75" s="31" t="s">
         <v>82</v>
@@ -5765,7 +5765,7 @@
         <v>61</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C76" s="27" t="s">
         <v>83</v>
@@ -5784,7 +5784,7 @@
         <v>0.0902777777777778</v>
       </c>
       <c r="H76" s="30" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I76" s="31" t="s">
         <v>79</v>
@@ -5793,13 +5793,13 @@
         <v>174486</v>
       </c>
       <c r="K76" s="31" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L76" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M76" s="31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="N76" s="31" t="s">
         <v>82</v>
@@ -5810,7 +5810,7 @@
         <v>61</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C77" s="27" t="s">
         <v>9</v>
@@ -5829,7 +5829,7 @@
         <v>0.195833333333333</v>
       </c>
       <c r="H77" s="30" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I77" s="31" t="s">
         <v>79</v>
@@ -5838,13 +5838,13 @@
         <v>174555</v>
       </c>
       <c r="K77" s="31" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="L77" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M77" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N77" s="31" t="s">
         <v>95</v>
@@ -5855,7 +5855,7 @@
         <v>61</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C78" s="27" t="s">
         <v>9</v>
@@ -5874,7 +5874,7 @@
         <v>0.109027777777778</v>
       </c>
       <c r="H78" s="30" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I78" s="31" t="s">
         <v>79</v>
@@ -5883,13 +5883,13 @@
         <v>174555</v>
       </c>
       <c r="K78" s="31" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="L78" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M78" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N78" s="31" t="s">
         <v>95</v>
@@ -5900,7 +5900,7 @@
         <v>61</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C79" s="27" t="s">
         <v>9</v>
@@ -5919,7 +5919,7 @@
         <v>0.0430555555555556</v>
       </c>
       <c r="H79" s="32" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="I79" s="31" t="s">
         <v>79</v>
@@ -5934,7 +5934,7 @@
         <v>3</v>
       </c>
       <c r="M79" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N79" s="31" t="s">
         <v>95</v>
@@ -5945,7 +5945,7 @@
         <v>61</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C80" s="27" t="s">
         <v>11</v>
@@ -5964,7 +5964,7 @@
         <v>0.0840277777777778</v>
       </c>
       <c r="H80" s="30" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I80" s="31" t="s">
         <v>79</v>
@@ -5979,7 +5979,7 @@
         <v>3</v>
       </c>
       <c r="M80" s="31" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="N80" s="31" t="s">
         <v>95</v>
@@ -5990,7 +5990,7 @@
         <v>61</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C81" s="27" t="s">
         <v>118</v>
@@ -6009,7 +6009,7 @@
         <v>0.0743055555555556</v>
       </c>
       <c r="H81" s="30" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I81" s="31" t="s">
         <v>79</v>
@@ -6018,13 +6018,13 @@
         <v>174616</v>
       </c>
       <c r="K81" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>8</v>
       </c>
       <c r="M81" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="N81" s="31" t="s">
         <v>82</v>
@@ -6035,7 +6035,7 @@
         <v>61</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C82" s="27" t="s">
         <v>113</v>
@@ -6054,7 +6054,7 @@
         <v>0.0854166666666667</v>
       </c>
       <c r="H82" s="30" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="I82" s="31" t="s">
         <v>79</v>
@@ -6063,13 +6063,13 @@
         <v>174708</v>
       </c>
       <c r="K82" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L82" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M82" s="31" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N82" s="31" t="s">
         <v>82</v>
@@ -6080,7 +6080,7 @@
         <v>61</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C83" s="27" t="s">
         <v>77</v>
@@ -6099,7 +6099,7 @@
         <v>0.0465277777777778</v>
       </c>
       <c r="H83" s="30" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I83" s="31" t="s">
         <v>89</v>
@@ -6108,13 +6108,13 @@
         <v>174783</v>
       </c>
       <c r="K83" s="31" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M83" s="31" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="N83" s="31" t="s">
         <v>82</v>
@@ -6125,7 +6125,7 @@
         <v>61</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C84" s="27" t="s">
         <v>130</v>
@@ -6144,7 +6144,7 @@
         <v>0.0402777777777778</v>
       </c>
       <c r="H84" s="30" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I84" s="31" t="s">
         <v>79</v>
@@ -6153,13 +6153,13 @@
         <v>174872</v>
       </c>
       <c r="K84" s="31" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="L84" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M84" s="31" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="N84" s="31" t="s">
         <v>82</v>
@@ -6170,7 +6170,7 @@
         <v>61</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C85" s="27" t="s">
         <v>83</v>
@@ -6189,7 +6189,7 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="H85" s="30" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="I85" s="31" t="s">
         <v>120</v>
@@ -6198,13 +6198,13 @@
         <v>174936</v>
       </c>
       <c r="K85" s="31" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L85" s="31" t="n">
         <v>1</v>
       </c>
       <c r="M85" s="31" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="N85" s="31" t="s">
         <v>82</v>
@@ -6215,7 +6215,7 @@
         <v>61</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C86" s="27" t="s">
         <v>9</v>
@@ -6234,7 +6234,7 @@
         <v>0.211111111111111</v>
       </c>
       <c r="H86" s="32" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I86" s="31" t="s">
         <v>79</v>
@@ -6243,13 +6243,13 @@
         <v>175066</v>
       </c>
       <c r="K86" s="31" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="L86" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M86" s="31" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="N86" s="31" t="s">
         <v>95</v>
@@ -6260,7 +6260,7 @@
         <v>61</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C87" s="27" t="s">
         <v>11</v>
@@ -6279,7 +6279,7 @@
         <v>0.0659722222222222</v>
       </c>
       <c r="H87" s="30" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I87" s="31" t="s">
         <v>89</v>
@@ -6288,13 +6288,13 @@
         <v>175070</v>
       </c>
       <c r="K87" s="31" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L87" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M87" s="31" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="N87" s="31" t="s">
         <v>95</v>
@@ -6305,7 +6305,7 @@
         <v>61</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C88" s="27" t="s">
         <v>11</v>
@@ -6324,7 +6324,7 @@
         <v>0.0798611111111111</v>
       </c>
       <c r="H88" s="30" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="I88" s="31" t="s">
         <v>79</v>
@@ -6333,13 +6333,13 @@
         <v>175070</v>
       </c>
       <c r="K88" s="31" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L88" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M88" s="31" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="N88" s="31" t="s">
         <v>95</v>
@@ -6350,7 +6350,7 @@
         <v>51</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C89" s="27" t="s">
         <v>113</v>
@@ -6369,7 +6369,7 @@
         <v>0.0736111111111111</v>
       </c>
       <c r="H89" s="32" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="I89" s="31" t="s">
         <v>173</v>
@@ -6378,13 +6378,13 @@
         <v>174216</v>
       </c>
       <c r="K89" s="31" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L89" s="31" t="n">
         <v>4</v>
       </c>
       <c r="M89" s="31" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N89" s="31" t="s">
         <v>82</v>
@@ -6395,7 +6395,7 @@
         <v>51</v>
       </c>
       <c r="B90" s="26" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C90" s="27" t="s">
         <v>118</v>
@@ -6414,7 +6414,7 @@
         <v>0.0659722222222222</v>
       </c>
       <c r="H90" s="30" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I90" s="31" t="s">
         <v>173</v>
@@ -6423,13 +6423,13 @@
         <v>174577</v>
       </c>
       <c r="K90" s="31" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L90" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M90" s="31" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="N90" s="31" t="s">
         <v>82</v>
@@ -6440,7 +6440,7 @@
         <v>51</v>
       </c>
       <c r="B91" s="26" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C91" s="27" t="s">
         <v>118</v>
@@ -6459,7 +6459,7 @@
         <v>0.05625</v>
       </c>
       <c r="H91" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I91" s="31" t="s">
         <v>173</v>
@@ -6468,13 +6468,13 @@
         <v>175122</v>
       </c>
       <c r="K91" s="31" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="L91" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M91" s="31" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="N91" s="31" t="s">
         <v>82</v>
@@ -6485,7 +6485,7 @@
         <v>51</v>
       </c>
       <c r="B92" s="26" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C92" s="27" t="s">
         <v>113</v>
@@ -6504,7 +6504,7 @@
         <v>0.0659722222222222</v>
       </c>
       <c r="H92" s="30" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="I92" s="31" t="s">
         <v>173</v>
@@ -6513,13 +6513,13 @@
         <v>175166</v>
       </c>
       <c r="K92" s="31" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="L92" s="31" t="n">
         <v>2</v>
       </c>
       <c r="M92" s="31" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="N92" s="31" t="s">
         <v>82</v>
@@ -6530,7 +6530,7 @@
         <v>56</v>
       </c>
       <c r="B93" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C93" s="27" t="s">
         <v>130</v>
@@ -6549,7 +6549,7 @@
         <v>0.104166666666667</v>
       </c>
       <c r="H93" s="32" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I93" s="31" t="s">
         <v>79</v>
@@ -6564,7 +6564,7 @@
         <v>3</v>
       </c>
       <c r="M93" s="31" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="N93" s="31" t="s">
         <v>82</v>
@@ -6575,7 +6575,7 @@
         <v>56</v>
       </c>
       <c r="B94" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C94" s="27" t="s">
         <v>83</v>
@@ -6594,7 +6594,7 @@
         <v>0.208333333333333</v>
       </c>
       <c r="H94" s="30" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I94" s="31" t="s">
         <v>79</v>
@@ -6603,13 +6603,13 @@
         <v>174030</v>
       </c>
       <c r="K94" s="31" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L94" s="31" t="n">
         <v>11</v>
       </c>
       <c r="M94" s="31" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="N94" s="31" t="s">
         <v>87</v>
@@ -6620,7 +6620,7 @@
         <v>56</v>
       </c>
       <c r="B95" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C95" s="27" t="s">
         <v>83</v>
@@ -6639,7 +6639,7 @@
         <v>0.177777777777778</v>
       </c>
       <c r="H95" s="30" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="I95" s="31" t="s">
         <v>89</v>
@@ -6648,13 +6648,13 @@
         <v>174030</v>
       </c>
       <c r="K95" s="31" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="L95" s="31" t="n">
         <v>11</v>
       </c>
       <c r="M95" s="31" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="N95" s="31" t="s">
         <v>87</v>
@@ -6665,7 +6665,7 @@
         <v>56</v>
       </c>
       <c r="B96" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C96" s="27" t="s">
         <v>9</v>
@@ -6684,22 +6684,22 @@
         <v>0.170833333333333</v>
       </c>
       <c r="H96" s="32" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="I96" s="31" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J96" s="31" t="n">
         <v>174054</v>
       </c>
       <c r="K96" s="31" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="L96" s="31" t="n">
         <v>5</v>
       </c>
       <c r="M96" s="31" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N96" s="31" t="s">
         <v>95</v>
@@ -6710,7 +6710,7 @@
         <v>56</v>
       </c>
       <c r="B97" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C97" s="27" t="s">
         <v>9</v>
@@ -6729,7 +6729,7 @@
         <v>0.0416666666666667</v>
       </c>
       <c r="H97" s="32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I97" s="31" t="s">
         <v>173</v>
@@ -6738,13 +6738,13 @@
         <v>174054</v>
       </c>
       <c r="K97" s="31" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="L97" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M97" s="31" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N97" s="31" t="s">
         <v>95</v>
@@ -6755,7 +6755,7 @@
         <v>56</v>
       </c>
       <c r="B98" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C98" s="27" t="s">
         <v>9</v>
@@ -6774,7 +6774,7 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="H98" s="30" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="I98" s="31" t="s">
         <v>79</v>
@@ -6789,7 +6789,7 @@
         <v>3</v>
       </c>
       <c r="M98" s="31" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N98" s="31" t="s">
         <v>95</v>
@@ -6800,7 +6800,7 @@
         <v>56</v>
       </c>
       <c r="B99" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C99" s="27" t="s">
         <v>11</v>
@@ -6819,22 +6819,22 @@
         <v>0.152777777777778</v>
       </c>
       <c r="H99" s="32" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="I99" s="31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J99" s="31" t="n">
         <v>174076</v>
       </c>
       <c r="K99" s="31" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L99" s="31" t="n">
         <v>7</v>
       </c>
       <c r="M99" s="31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="N99" s="31" t="s">
         <v>95</v>
@@ -6845,7 +6845,7 @@
         <v>56</v>
       </c>
       <c r="B100" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C100" s="27" t="s">
         <v>11</v>
@@ -6864,22 +6864,22 @@
         <v>0.118055555555556</v>
       </c>
       <c r="H100" s="30" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="I100" s="31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J100" s="31" t="n">
         <v>174076</v>
       </c>
       <c r="K100" s="31" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="L100" s="31" t="n">
         <v>7</v>
       </c>
       <c r="M100" s="31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="N100" s="31" t="s">
         <v>95</v>
@@ -6890,7 +6890,7 @@
         <v>56</v>
       </c>
       <c r="B101" s="26" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C101" s="27" t="s">
         <v>11</v>
@@ -6909,7 +6909,7 @@
         <v>0.104166666666667</v>
       </c>
       <c r="H101" s="32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="I101" s="31" t="s">
         <v>79</v>
@@ -6918,13 +6918,13 @@
         <v>174076</v>
       </c>
       <c r="K101" s="31" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L101" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M101" s="31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="N101" s="31" t="s">
         <v>95</v>
@@ -6935,7 +6935,7 @@
         <v>56</v>
       </c>
       <c r="B102" s="26" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C102" s="27" t="s">
         <v>113</v>
@@ -6954,7 +6954,7 @@
         <v>0.0416666666666667</v>
       </c>
       <c r="H102" s="32" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="I102" s="31" t="s">
         <v>79</v>
@@ -6963,13 +6963,13 @@
         <v>174727</v>
       </c>
       <c r="K102" s="31" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="L102" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M102" s="31" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="N102" s="31" t="s">
         <v>82</v>
@@ -6980,7 +6980,7 @@
         <v>60</v>
       </c>
       <c r="B103" s="26" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C103" s="27" t="s">
         <v>113</v>
@@ -6999,7 +6999,7 @@
         <v>0.0555555555555556</v>
       </c>
       <c r="H103" s="32" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="I103" s="31" t="s">
         <v>89</v>
@@ -7008,13 +7008,13 @@
         <v>174710</v>
       </c>
       <c r="K103" s="31" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="L103" s="31" t="n">
         <v>1</v>
       </c>
       <c r="M103" s="31" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N103" s="31" t="s">
         <v>82</v>
@@ -7025,7 +7025,7 @@
         <v>60</v>
       </c>
       <c r="B104" s="26" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C104" s="27" t="s">
         <v>113</v>
@@ -7044,7 +7044,7 @@
         <v>0.0798611111111111</v>
       </c>
       <c r="H104" s="32" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I104" s="31" t="s">
         <v>79</v>
@@ -7053,13 +7053,13 @@
         <v>175158</v>
       </c>
       <c r="K104" s="31" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="L104" s="31" t="n">
         <v>3</v>
       </c>
       <c r="M104" s="31" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="N104" s="31" t="s">
         <v>82</v>
@@ -7070,7 +7070,7 @@
         <v>62</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C105" s="27" t="s">
         <v>130</v>
@@ -7089,7 +7089,7 @@
         <v>0.0618055555555556</v>
       </c>
       <c r="H105" s="30" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="I105" s="31" t="s">
         <v>79</v>
@@ -7104,7 +7104,7 @@
         <v>3</v>
       </c>
       <c r="M105" s="31" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="N105" s="31" t="s">
         <v>82</v>
@@ -7115,7 +7115,7 @@
         <v>62</v>
       </c>
       <c r="B106" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C106" s="27" t="s">
         <v>83</v>
@@ -7134,7 +7134,7 @@
         <v>0.181944444444444</v>
       </c>
       <c r="H106" s="30" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I106" s="31" t="s">
         <v>173</v>
@@ -7143,7 +7143,7 @@
         <v>174080</v>
       </c>
       <c r="K106" s="31" t="s">
-        <v>388</v>
+        <v>247</v>
       </c>
       <c r="L106" s="31" t="n">
         <v>5</v>
@@ -7160,7 +7160,7 @@
         <v>62</v>
       </c>
       <c r="B107" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C107" s="27" t="s">
         <v>83</v>
@@ -7205,7 +7205,7 @@
         <v>62</v>
       </c>
       <c r="B108" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C108" s="27" t="s">
         <v>9</v>
@@ -7250,7 +7250,7 @@
         <v>62</v>
       </c>
       <c r="B109" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C109" s="27" t="s">
         <v>11</v>

</xml_diff>